<commit_message>
fix: change server port to 8080 to prevent BindException on Linux and align with client configuration
</commit_message>
<xml_diff>
--- a/enunciado/Justificaciones.xlsx
+++ b/enunciado/Justificaciones.xlsx
@@ -1969,6 +1969,86 @@
         <v>83</v>
       </c>
     </row>
+    <row r="1002">
+      <c r="A1002" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1002" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1002" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1002" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1002" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1002" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1003" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1003" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1003" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1003" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1003" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1004" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1004" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1004" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1004" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1004" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1005" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1005" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1005" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1005" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1005" t="s">
+        <v>83</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>